<commit_message>
Fix nx import, unify naming to DeepWalk-SSP, add PCA stats, update all results
- Fix NameError in add_baselines.py: move networkx import to module level
- Rename "DeepWalk Embeddings" → "DeepWalk-SSP" in all plots and titles
- Add Step 5b: Wilcoxon signed-rank test for DeepWalk vs PCA+KMeans
- Add exp_statistical_analysis_pca.json with per-course and aggregate results
- Re-run full experiment suite; update all result files and figures
- Update README.md with current numbers and Springer template reference

🤖 Generated with Codebuff
Co-Authored-By: Codebuff <noreply@codebuff.com>
</commit_message>
<xml_diff>
--- a/results/baseline_pca_kmeans.xlsx
+++ b/results/baseline_pca_kmeans.xlsx
@@ -1,13 +1,13 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <workbookProtection/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" tabRatio="600" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
@@ -509,7 +509,7 @@
         <v>0.5862144827842712</v>
       </c>
       <c r="J2" t="n">
-        <v>0.8443555000703782</v>
+        <v>0.02248180005699396</v>
       </c>
     </row>
     <row r="3">
@@ -541,7 +541,7 @@
         <v>0.5674307942390442</v>
       </c>
       <c r="J3" t="n">
-        <v>0.01997449994087219</v>
+        <v>0.02204660000279546</v>
       </c>
     </row>
     <row r="4">
@@ -573,7 +573,7 @@
         <v>0.5507810115814209</v>
       </c>
       <c r="J4" t="n">
-        <v>0.02056430000811815</v>
+        <v>0.02378249983303249</v>
       </c>
     </row>
     <row r="5">
@@ -605,7 +605,7 @@
         <v>0.5601266622543335</v>
       </c>
       <c r="J5" t="n">
-        <v>0.02840310009196401</v>
+        <v>0.02290660003200173</v>
       </c>
     </row>
     <row r="6">
@@ -637,7 +637,7 @@
         <v>0.6120653748512268</v>
       </c>
       <c r="J6" t="n">
-        <v>0.01918089995160699</v>
+        <v>0.02365999994799495</v>
       </c>
     </row>
     <row r="7">
@@ -669,7 +669,7 @@
         <v>0.5969101786613464</v>
       </c>
       <c r="J7" t="n">
-        <v>0.02316640014760196</v>
+        <v>0.0234574000351131</v>
       </c>
     </row>
   </sheetData>

</xml_diff>